<commit_message>
Add residuals, appraisal ratio, and Word answers document
Excel updates:
- Added CAPM residuals columns (Q, R) in Monthly Returns sheet
- Added Std Dev of Residuals and Appraisal Ratio in CAPM Regression sheet

Word document answers all Chapter 11 & 12 questions:
- Ch11 a.1: Statistical significance of alpha and beta
- Ch11 a.2: Interpretation of alpha and beta
- Ch11 a.3: R-squared comparison (VFIAX > AAPL)
- Ch11 b.1: What appraisal ratio measures
- Ch11 b.2: Appraisal ratio calculations
- Ch11 b.3: Why appraisal ratio used more for mutual funds
- Ch12 1.a-d: Four-factor model analysis

https://claude.ai/code/session_01UFgKuhfYfoTRdFuN7kHBHu
</commit_message>
<xml_diff>
--- a/Finance_Homework.xlsx
+++ b/Finance_Homework.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Monthly Returns" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Descriptive Statistics" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="CAPM Regression" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="FF4 Regression" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Returns" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Descriptive Statistics" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAPM Regression" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FF4 Regression" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -467,25 +467,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P65"/>
+  <dimension ref="A1:R65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="15" customWidth="1" min="11" max="11"/>
     <col width="17" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -577,6 +579,16 @@
           <t>Mom</t>
         </is>
       </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>AAPL CAPM Resid</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>VFIAX CAPM Resid</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
@@ -662,6 +674,12 @@
       <c r="P5" s="6" t="n">
         <v>-0.0612</v>
       </c>
+      <c r="Q5" s="6" t="n">
+        <v>-0.02896020649212365</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>0.008075318148560759</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
@@ -718,6 +736,12 @@
       <c r="P6" s="6" t="n">
         <v>0.0123</v>
       </c>
+      <c r="Q6" s="6" t="n">
+        <v>0.01934905946307464</v>
+      </c>
+      <c r="R6" s="6" t="n">
+        <v>0.007310301032694942</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
@@ -774,6 +798,12 @@
       <c r="P7" s="6" t="n">
         <v>0.005600000000000001</v>
       </c>
+      <c r="Q7" s="6" t="n">
+        <v>-0.0593393559821066</v>
+      </c>
+      <c r="R7" s="6" t="n">
+        <v>0.003109524512750906</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
@@ -830,6 +860,12 @@
       <c r="P8" s="6" t="n">
         <v>0.0207</v>
       </c>
+      <c r="Q8" s="6" t="n">
+        <v>0.06771826125081251</v>
+      </c>
+      <c r="R8" s="6" t="n">
+        <v>-0.008056892876751785</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
@@ -886,6 +922,12 @@
       <c r="P9" s="6" t="n">
         <v>-0.0218</v>
       </c>
+      <c r="Q9" s="6" t="n">
+        <v>0.04660640045901524</v>
+      </c>
+      <c r="R9" s="6" t="n">
+        <v>0.01308261452428771</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
@@ -942,6 +984,12 @@
       <c r="P10" s="6" t="n">
         <v>0.0263</v>
       </c>
+      <c r="Q10" s="6" t="n">
+        <v>0.005466308902687046</v>
+      </c>
+      <c r="R10" s="6" t="n">
+        <v>0.0004630477922934716</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
@@ -998,6 +1046,12 @@
       <c r="P11" s="6" t="n">
         <v>0.0139</v>
       </c>
+      <c r="Q11" s="6" t="n">
+        <v>-0.02370074577106621</v>
+      </c>
+      <c r="R11" s="6" t="n">
+        <v>-0.007111752511926091</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
@@ -1054,6 +1108,12 @@
       <c r="P12" s="6" t="n">
         <v>0.0332</v>
       </c>
+      <c r="Q12" s="6" t="n">
+        <v>-0.0161663600762522</v>
+      </c>
+      <c r="R12" s="6" t="n">
+        <v>0.007174500103029308</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
@@ -1110,6 +1170,12 @@
       <c r="P13" s="6" t="n">
         <v>0.009599999999999999</v>
       </c>
+      <c r="Q13" s="6" t="n">
+        <v>0.116329027110048</v>
+      </c>
+      <c r="R13" s="6" t="n">
+        <v>0.007712067659851159</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
@@ -1166,6 +1232,12 @@
       <c r="P14" s="6" t="n">
         <v>-0.0239</v>
       </c>
+      <c r="Q14" s="6" t="n">
+        <v>0.03715378709554483</v>
+      </c>
+      <c r="R14" s="6" t="n">
+        <v>0.008151639087974123</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
@@ -1222,6 +1294,12 @@
       <c r="P15" s="6" t="n">
         <v>-0.0242</v>
       </c>
+      <c r="Q15" s="6" t="n">
+        <v>0.04600796727245694</v>
+      </c>
+      <c r="R15" s="6" t="n">
+        <v>0.01151734885452275</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
@@ -1278,6 +1356,12 @@
       <c r="P16" s="6" t="n">
         <v>0.0166</v>
       </c>
+      <c r="Q16" s="6" t="n">
+        <v>-0.0349562061825185</v>
+      </c>
+      <c r="R16" s="6" t="n">
+        <v>-0.008350431778571449</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
@@ -1334,6 +1418,12 @@
       <c r="P17" s="6" t="n">
         <v>0.0294</v>
       </c>
+      <c r="Q17" s="6" t="n">
+        <v>0.02186947052768291</v>
+      </c>
+      <c r="R17" s="6" t="n">
+        <v>0.002366395155027873</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
@@ -1390,6 +1480,12 @@
       <c r="P18" s="6" t="n">
         <v>0.05</v>
       </c>
+      <c r="Q18" s="6" t="n">
+        <v>-0.0007319477765609372</v>
+      </c>
+      <c r="R18" s="6" t="n">
+        <v>0.007728581871668957</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
@@ -1446,6 +1542,12 @@
       <c r="P19" s="6" t="n">
         <v>0.0254</v>
       </c>
+      <c r="Q19" s="6" t="n">
+        <v>-0.05658582987561828</v>
+      </c>
+      <c r="R19" s="6" t="n">
+        <v>0.003941839286208193</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
@@ -1502,6 +1604,12 @@
       <c r="P20" s="6" t="n">
         <v>0.0109</v>
       </c>
+      <c r="Q20" s="6" t="n">
+        <v>0.004939786197488569</v>
+      </c>
+      <c r="R20" s="6" t="n">
+        <v>-0.004900070223386205</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
@@ -1558,6 +1666,12 @@
       <c r="P21" s="6" t="n">
         <v>-0.0436</v>
       </c>
+      <c r="Q21" s="6" t="n">
+        <v>0.08165863842367754</v>
+      </c>
+      <c r="R21" s="6" t="n">
+        <v>0.0004260673371504625</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n">
@@ -1614,6 +1728,12 @@
       <c r="P22" s="6" t="n">
         <v>0.0185</v>
       </c>
+      <c r="Q22" s="6" t="n">
+        <v>0.001756826372491568</v>
+      </c>
+      <c r="R22" s="6" t="n">
+        <v>-0.006392439682232971</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
@@ -1670,6 +1790,12 @@
       <c r="P23" s="6" t="n">
         <v>0.0367</v>
       </c>
+      <c r="Q23" s="6" t="n">
+        <v>-0.02602169782501856</v>
+      </c>
+      <c r="R23" s="6" t="n">
+        <v>-0.006716598316649419</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
@@ -1726,6 +1852,12 @@
       <c r="P24" s="6" t="n">
         <v>0.039</v>
       </c>
+      <c r="Q24" s="6" t="n">
+        <v>0.01943255457899207</v>
+      </c>
+      <c r="R24" s="6" t="n">
+        <v>0.005009973257944028</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
@@ -1782,6 +1914,12 @@
       <c r="P25" s="6" t="n">
         <v>-0.017</v>
       </c>
+      <c r="Q25" s="6" t="n">
+        <v>-0.09123116405911633</v>
+      </c>
+      <c r="R25" s="6" t="n">
+        <v>0.006160030032779588</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n">
@@ -1838,6 +1976,12 @@
       <c r="P26" s="6" t="n">
         <v>0.0491</v>
       </c>
+      <c r="Q26" s="6" t="n">
+        <v>-0.0600295595890652</v>
+      </c>
+      <c r="R26" s="6" t="n">
+        <v>-0.003365086060545273</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n">
@@ -1894,6 +2038,12 @@
       <c r="P27" s="6" t="n">
         <v>-0.1617</v>
       </c>
+      <c r="Q27" s="6" t="n">
+        <v>0.03238376727353851</v>
+      </c>
+      <c r="R27" s="6" t="n">
+        <v>-0.00175723693871517</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n">
@@ -1950,6 +2100,12 @@
       <c r="P28" s="6" t="n">
         <v>0.005500000000000001</v>
       </c>
+      <c r="Q28" s="6" t="n">
+        <v>0.0416114308752388</v>
+      </c>
+      <c r="R28" s="6" t="n">
+        <v>-0.003397558632274599</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n">
@@ -2006,6 +2162,12 @@
       <c r="P29" s="6" t="n">
         <v>-0.0235</v>
       </c>
+      <c r="Q29" s="6" t="n">
+        <v>0.08629685665677259</v>
+      </c>
+      <c r="R29" s="6" t="n">
+        <v>0.003540647802456717</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n">
@@ -2062,6 +2224,12 @@
       <c r="P30" s="6" t="n">
         <v>0.0176</v>
       </c>
+      <c r="Q30" s="6" t="n">
+        <v>0.01481318939114958</v>
+      </c>
+      <c r="R30" s="6" t="n">
+        <v>0.009206302605114791</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n">
@@ -2118,6 +2286,12 @@
       <c r="P31" s="6" t="n">
         <v>-0.008800000000000001</v>
       </c>
+      <c r="Q31" s="6" t="n">
+        <v>0.03332792829357033</v>
+      </c>
+      <c r="R31" s="6" t="n">
+        <v>-0.003524635084375526</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n">
@@ -2174,6 +2348,12 @@
       <c r="P32" s="6" t="n">
         <v>-0.0269</v>
       </c>
+      <c r="Q32" s="6" t="n">
+        <v>0.01880136084599558</v>
+      </c>
+      <c r="R32" s="6" t="n">
+        <v>-0.006705560462820948</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n">
@@ -2230,6 +2410,12 @@
       <c r="P33" s="6" t="n">
         <v>-0.0406</v>
       </c>
+      <c r="Q33" s="6" t="n">
+        <v>-0.03001637985244961</v>
+      </c>
+      <c r="R33" s="6" t="n">
+        <v>-0.0009390695330546775</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="n">
@@ -2286,6 +2472,12 @@
       <c r="P34" s="6" t="n">
         <v>0.0378</v>
       </c>
+      <c r="Q34" s="6" t="n">
+        <v>-0.02702873705702609</v>
+      </c>
+      <c r="R34" s="6" t="n">
+        <v>0.001974188963400306</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n">
@@ -2342,6 +2534,12 @@
       <c r="P35" s="6" t="n">
         <v>0.0033</v>
       </c>
+      <c r="Q35" s="6" t="n">
+        <v>-0.03992290297318975</v>
+      </c>
+      <c r="R35" s="6" t="n">
+        <v>-0.004889549647456762</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n">
@@ -2398,6 +2596,12 @@
       <c r="P36" s="6" t="n">
         <v>0.0167</v>
       </c>
+      <c r="Q36" s="6" t="n">
+        <v>0.02228517685841032</v>
+      </c>
+      <c r="R36" s="6" t="n">
+        <v>0.008147991659174146</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="n">
@@ -2454,6 +2658,12 @@
       <c r="P37" s="6" t="n">
         <v>0.0256</v>
       </c>
+      <c r="Q37" s="6" t="n">
+        <v>0.009084457687413561</v>
+      </c>
+      <c r="R37" s="6" t="n">
+        <v>-0.001618330165148146</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n">
@@ -2510,6 +2720,12 @@
       <c r="P38" s="6" t="n">
         <v>-0.0553</v>
       </c>
+      <c r="Q38" s="6" t="n">
+        <v>-0.04520762056218623</v>
+      </c>
+      <c r="R38" s="6" t="n">
+        <v>-0.01190724812383836</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="n">
@@ -2566,6 +2782,12 @@
       <c r="P39" s="6" t="n">
         <v>0.0542</v>
       </c>
+      <c r="Q39" s="6" t="n">
+        <v>-0.05878297606544287</v>
+      </c>
+      <c r="R39" s="6" t="n">
+        <v>0.008159583938603682</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="n">
@@ -2622,6 +2844,12 @@
       <c r="P40" s="6" t="n">
         <v>0.049</v>
       </c>
+      <c r="Q40" s="6" t="n">
+        <v>-0.08215056330929543</v>
+      </c>
+      <c r="R40" s="6" t="n">
+        <v>-0.001742967782112276</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="n">
@@ -2678,6 +2906,12 @@
       <c r="P41" s="6" t="n">
         <v>-0.0032</v>
       </c>
+      <c r="Q41" s="6" t="n">
+        <v>-0.08874939240583832</v>
+      </c>
+      <c r="R41" s="6" t="n">
+        <v>-0.004326613558199185</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="n">
@@ -2734,6 +2968,12 @@
       <c r="P42" s="6" t="n">
         <v>-0.0043</v>
       </c>
+      <c r="Q42" s="6" t="n">
+        <v>0.03419021731067522</v>
+      </c>
+      <c r="R42" s="6" t="n">
+        <v>0.00245869134143361</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="n">
@@ -2790,6 +3030,12 @@
       <c r="P43" s="6" t="n">
         <v>-0.0016</v>
       </c>
+      <c r="Q43" s="6" t="n">
+        <v>0.07407019172786297</v>
+      </c>
+      <c r="R43" s="6" t="n">
+        <v>0.001564669761153582</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="n">
@@ -2846,6 +3092,12 @@
       <c r="P44" s="6" t="n">
         <v>0.008500000000000001</v>
       </c>
+      <c r="Q44" s="6" t="n">
+        <v>0.05896197483977118</v>
+      </c>
+      <c r="R44" s="6" t="n">
+        <v>-0.0004391514533749578</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="n">
@@ -2902,6 +3154,12 @@
       <c r="P45" s="6" t="n">
         <v>-0.0235</v>
       </c>
+      <c r="Q45" s="6" t="n">
+        <v>0.03288178102397946</v>
+      </c>
+      <c r="R45" s="6" t="n">
+        <v>-0.001694183578875659</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="n">
@@ -2958,6 +3216,12 @@
       <c r="P46" s="6" t="n">
         <v>0.0481</v>
       </c>
+      <c r="Q46" s="6" t="n">
+        <v>0.005203274551998524</v>
+      </c>
+      <c r="R46" s="6" t="n">
+        <v>0.002762864946941387</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="n">
@@ -3014,6 +3278,12 @@
       <c r="P47" s="6" t="n">
         <v>-0.0062</v>
       </c>
+      <c r="Q47" s="6" t="n">
+        <v>-0.00774718401403016</v>
+      </c>
+      <c r="R47" s="6" t="n">
+        <v>-0.003713936447603317</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n">
@@ -3070,6 +3340,12 @@
       <c r="P48" s="6" t="n">
         <v>0.03</v>
       </c>
+      <c r="Q48" s="6" t="n">
+        <v>-0.0276807377969926</v>
+      </c>
+      <c r="R48" s="6" t="n">
+        <v>-0.0009313956164887487</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="n">
@@ -3126,6 +3402,12 @@
       <c r="P49" s="6" t="n">
         <v>0.01</v>
       </c>
+      <c r="Q49" s="6" t="n">
+        <v>-0.02680359919663823</v>
+      </c>
+      <c r="R49" s="6" t="n">
+        <v>-0.01024967213539595</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="n">
@@ -3182,6 +3464,12 @@
       <c r="P50" s="6" t="n">
         <v>-0.003</v>
       </c>
+      <c r="Q50" s="6" t="n">
+        <v>0.08242239589847414</v>
+      </c>
+      <c r="R50" s="6" t="n">
+        <v>-0.0002489464485813803</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="n">
@@ -3238,6 +3526,12 @@
       <c r="P51" s="6" t="n">
         <v>0.009599999999999999</v>
       </c>
+      <c r="Q51" s="6" t="n">
+        <v>-0.09521220328475762</v>
+      </c>
+      <c r="R51" s="6" t="n">
+        <v>-0.00113342911332703</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="n">
@@ -3294,6 +3588,12 @@
       <c r="P52" s="6" t="n">
         <v>-0.008100000000000001</v>
       </c>
+      <c r="Q52" s="6" t="n">
+        <v>0.04345828035031446</v>
+      </c>
+      <c r="R52" s="6" t="n">
+        <v>0.006808882021098431</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="n">
@@ -3350,6 +3650,12 @@
       <c r="P53" s="6" t="n">
         <v>-0.0284</v>
       </c>
+      <c r="Q53" s="6" t="n">
+        <v>-0.019714197144946</v>
+      </c>
+      <c r="R53" s="6" t="n">
+        <v>-0.0008599689955759091</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="n">
@@ -3406,6 +3712,12 @@
       <c r="P54" s="6" t="n">
         <v>0.04969999999999999</v>
       </c>
+      <c r="Q54" s="6" t="n">
+        <v>-0.04193617938623419</v>
+      </c>
+      <c r="R54" s="6" t="n">
+        <v>0.0005032740708776056</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="n">
@@ -3462,6 +3774,12 @@
       <c r="P55" s="6" t="n">
         <v>0.0221</v>
       </c>
+      <c r="Q55" s="6" t="n">
+        <v>-0.127364363698349</v>
+      </c>
+      <c r="R55" s="6" t="n">
+        <v>-0.001558809813728364</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="n">
@@ -3518,6 +3836,12 @@
       <c r="P56" s="6" t="n">
         <v>-0.0264</v>
       </c>
+      <c r="Q56" s="6" t="n">
+        <v>-0.03647554189115065</v>
+      </c>
+      <c r="R56" s="6" t="n">
+        <v>-0.004596760251053739</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="n">
@@ -3574,6 +3898,12 @@
       <c r="P57" s="6" t="n">
         <v>-0.0097</v>
       </c>
+      <c r="Q57" s="6" t="n">
+        <v>-0.01689738945319351</v>
+      </c>
+      <c r="R57" s="6" t="n">
+        <v>0.001674242026644887</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="n">
@@ -3630,6 +3960,12 @@
       <c r="P58" s="6" t="n">
         <v>-0.0354</v>
       </c>
+      <c r="Q58" s="6" t="n">
+        <v>0.09090483965320084</v>
+      </c>
+      <c r="R58" s="6" t="n">
+        <v>-0.002582189369196748</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="n">
@@ -3686,6 +4022,12 @@
       <c r="P59" s="6" t="n">
         <v>0.0463</v>
       </c>
+      <c r="Q59" s="6" t="n">
+        <v>0.05459035674430777</v>
+      </c>
+      <c r="R59" s="6" t="n">
+        <v>-0.004070720627130518</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="n">
@@ -3742,6 +4084,12 @@
       <c r="P60" s="6" t="n">
         <v>0.0027</v>
       </c>
+      <c r="Q60" s="6" t="n">
+        <v>0.03314583083122064</v>
+      </c>
+      <c r="R60" s="6" t="n">
+        <v>0.002357671145062554</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="n">
@@ -3798,6 +4146,12 @@
       <c r="P61" s="6" t="n">
         <v>-0.018</v>
       </c>
+      <c r="Q61" s="6" t="n">
+        <v>0.02569391496712614</v>
+      </c>
+      <c r="R61" s="6" t="n">
+        <v>-0.0001870451812073436</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="n">
@@ -3854,6 +4208,12 @@
       <c r="P62" s="6" t="n">
         <v>-0.024</v>
       </c>
+      <c r="Q62" s="6" t="n">
+        <v>-0.02770918314212299</v>
+      </c>
+      <c r="R62" s="6" t="n">
+        <v>-0.002947747445282775</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="n">
@@ -3910,6 +4270,12 @@
       <c r="P63" s="6" t="n">
         <v>0.0495</v>
       </c>
+      <c r="Q63" s="6" t="n">
+        <v>-0.06347606544089365</v>
+      </c>
+      <c r="R63" s="6" t="n">
+        <v>0.003369417498569482</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="n">
@@ -3951,6 +4317,12 @@
         <f>G64-H64</f>
         <v/>
       </c>
+      <c r="Q64" s="6" t="n">
+        <v>0.01404781852784766</v>
+      </c>
+      <c r="R64" s="6" t="n">
+        <v>-0.008511490353032676</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="n">
@@ -3992,10 +4364,16 @@
         <f>G65-H65</f>
         <v/>
       </c>
+      <c r="Q65" s="6" t="n">
+        <v>-0.01586484165865719</v>
+      </c>
+      <c r="R65" s="6" t="n">
+        <v>-0.01533018822936139</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A1:R1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4010,13 +4388,13 @@
   <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4530,11 +4908,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="3" customWidth="1" min="3" max="3"/>
     <col width="3" customWidth="1" min="4" max="4"/>
     <col width="3" customWidth="1" min="5" max="5"/>
@@ -4674,123 +5052,167 @@
         <v/>
       </c>
     </row>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Std Dev of Residuals</t>
+        </is>
+      </c>
+      <c r="B15" s="8">
+        <f>STDEV.S('Monthly Returns'!Q5:Q65)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Appraisal Ratio</t>
+        </is>
+      </c>
+      <c r="B16" s="8">
+        <f>B6/B15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
         <is>
           <t>VFIAX Market Model</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Statistic</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>Alpha (α)</t>
-        </is>
-      </c>
-      <c r="B19" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!K5:K65,'Monthly Returns'!M5:M65,TRUE,TRUE),1,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>Beta (β)</t>
-        </is>
-      </c>
-      <c r="B20" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!K5:K65,'Monthly Returns'!M5:M65,TRUE,TRUE),1,1)</f>
-        <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>R-squared</t>
+          <t>Alpha (α)</t>
         </is>
       </c>
       <c r="B21" s="8">
-        <f>RSQ('Monthly Returns'!K5:K65,'Monthly Returns'!M5:M65)</f>
+        <f>INDEX(LINEST('Monthly Returns'!K5:K65,'Monthly Returns'!M5:M65,TRUE,TRUE),1,2)</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>Std Error (α)</t>
+          <t>Beta (β)</t>
         </is>
       </c>
       <c r="B22" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!K5:K65,'Monthly Returns'!M5:M65,TRUE,TRUE),2,2)</f>
+        <f>INDEX(LINEST('Monthly Returns'!K5:K65,'Monthly Returns'!M5:M65,TRUE,TRUE),1,1)</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>Std Error (β)</t>
+          <t>R-squared</t>
         </is>
       </c>
       <c r="B23" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!K5:K65,'Monthly Returns'!M5:M65,TRUE,TRUE),2,1)</f>
+        <f>RSQ('Monthly Returns'!K5:K65,'Monthly Returns'!M5:M65)</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>t-stat (α)</t>
+          <t>Std Error (α)</t>
         </is>
       </c>
       <c r="B24" s="8">
-        <f>B19/B22</f>
+        <f>INDEX(LINEST('Monthly Returns'!K5:K65,'Monthly Returns'!M5:M65,TRUE,TRUE),2,2)</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>t-stat (β)</t>
+          <t>Std Error (β)</t>
         </is>
       </c>
       <c r="B25" s="8">
-        <f>B20/B23</f>
+        <f>INDEX(LINEST('Monthly Returns'!K5:K65,'Monthly Returns'!M5:M65,TRUE,TRUE),2,1)</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>F-statistic</t>
+          <t>t-stat (α)</t>
         </is>
       </c>
       <c r="B26" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!K5:K65,'Monthly Returns'!M5:M65,TRUE,TRUE),4,1)</f>
+        <f>B21/B24</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
+          <t>t-stat (β)</t>
+        </is>
+      </c>
+      <c r="B27" s="8">
+        <f>B22/B25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>F-statistic</t>
+        </is>
+      </c>
+      <c r="B28" s="8">
+        <f>INDEX(LINEST('Monthly Returns'!K5:K65,'Monthly Returns'!M5:M65,TRUE,TRUE),4,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
           <t>Observations</t>
         </is>
       </c>
-      <c r="B27" s="8">
+      <c r="B29" s="8">
         <f>COUNT('Monthly Returns'!K5:K65)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>Std Dev of Residuals</t>
+        </is>
+      </c>
+      <c r="B30" s="8">
+        <f>STDEV.S('Monthly Returns'!R5:R65)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>Appraisal Ratio</t>
+        </is>
+      </c>
+      <c r="B31" s="8">
+        <f>B21/B30</f>
         <v/>
       </c>
     </row>
@@ -4811,8 +5233,8 @@
   <dimension ref="A1:F45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="3" customWidth="1" min="3" max="3"/>
     <col width="3" customWidth="1" min="4" max="4"/>
     <col width="3" customWidth="1" min="5" max="5"/>
@@ -4822,7 +5244,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Fama-French 3-Factor + Momentum Regression</t>
+          <t>Fama-French 3-Factor + Momentum (Carhart 4-Factor) Regression</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Excel compatibility: replace LINEST formulas with computed values
- STDEV.S/VAR.S -> STDEV/VAR (fixes #NAME? in Descriptive Statistics)
- All CAPM & FF4 regression values now written as Python-computed numbers
  instead of LINEST/INDEX formulas (fixes #VALUE! errors)
- Fixes cascade errors in Annualized Std Dev and Sharpe Ratio

https://claude.ai/code/session_01UFgKuhfYfoTRdFuN7kHBHu
</commit_message>
<xml_diff>
--- a/Finance_Homework.xlsx
+++ b/Finance_Homework.xlsx
@@ -4511,27 +4511,27 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>STDEV.S('Monthly Returns'!E5:E65)</f>
+        <f>STDEV('Monthly Returns'!E5:E65)</f>
         <v/>
       </c>
       <c r="C6" s="5">
-        <f>STDEV.S('Monthly Returns'!F5:F65)</f>
+        <f>STDEV('Monthly Returns'!F5:F65)</f>
         <v/>
       </c>
       <c r="D6" s="5">
-        <f>STDEV.S('Monthly Returns'!G5:G65)</f>
+        <f>STDEV('Monthly Returns'!G5:G65)</f>
         <v/>
       </c>
       <c r="E6" s="5">
-        <f>STDEV.S('Monthly Returns'!J5:J65)</f>
+        <f>STDEV('Monthly Returns'!J5:J65)</f>
         <v/>
       </c>
       <c r="F6" s="5">
-        <f>STDEV.S('Monthly Returns'!K5:K65)</f>
+        <f>STDEV('Monthly Returns'!K5:K65)</f>
         <v/>
       </c>
       <c r="G6" s="5">
-        <f>STDEV.S('Monthly Returns'!L5:L65)</f>
+        <f>STDEV('Monthly Returns'!L5:L65)</f>
         <v/>
       </c>
     </row>
@@ -4542,27 +4542,27 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>VAR.S('Monthly Returns'!E5:E65)</f>
+        <f>VAR('Monthly Returns'!E5:E65)</f>
         <v/>
       </c>
       <c r="C7" s="5">
-        <f>VAR.S('Monthly Returns'!F5:F65)</f>
+        <f>VAR('Monthly Returns'!F5:F65)</f>
         <v/>
       </c>
       <c r="D7" s="5">
-        <f>VAR.S('Monthly Returns'!G5:G65)</f>
+        <f>VAR('Monthly Returns'!G5:G65)</f>
         <v/>
       </c>
       <c r="E7" s="5">
-        <f>VAR.S('Monthly Returns'!J5:J65)</f>
+        <f>VAR('Monthly Returns'!J5:J65)</f>
         <v/>
       </c>
       <c r="F7" s="5">
-        <f>VAR.S('Monthly Returns'!K5:K65)</f>
+        <f>VAR('Monthly Returns'!K5:K65)</f>
         <v/>
       </c>
       <c r="G7" s="5">
-        <f>VAR.S('Monthly Returns'!L5:L65)</f>
+        <f>VAR('Monthly Returns'!L5:L65)</f>
         <v/>
       </c>
     </row>
@@ -4908,7 +4908,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4959,9 +4959,8 @@
           <t>Alpha (α)</t>
         </is>
       </c>
-      <c r="B6" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!J5:J65,'Monthly Returns'!M5:M65,TRUE,TRUE),1,2)</f>
-        <v/>
+      <c r="B6" s="8" t="n">
+        <v>0.004043525400558397</v>
       </c>
     </row>
     <row r="7">
@@ -4970,9 +4969,8 @@
           <t>Beta (β)</t>
         </is>
       </c>
-      <c r="B7" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!J5:J65,'Monthly Returns'!M5:M65,TRUE,TRUE),1,1)</f>
-        <v/>
+      <c r="B7" s="8" t="n">
+        <v>1.067578224673151</v>
       </c>
     </row>
     <row r="8">
@@ -4981,9 +4979,8 @@
           <t>R-squared</t>
         </is>
       </c>
-      <c r="B8" s="8">
-        <f>RSQ('Monthly Returns'!J5:J65,'Monthly Returns'!M5:M65)</f>
-        <v/>
+      <c r="B8" s="8" t="n">
+        <v>0.4531008081301806</v>
       </c>
     </row>
     <row r="9">
@@ -4992,9 +4989,8 @@
           <t>Std Error (α)</t>
         </is>
       </c>
-      <c r="B9" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!J5:J65,'Monthly Returns'!M5:M65,TRUE,TRUE),2,2)</f>
-        <v/>
+      <c r="B9" s="8" t="n">
+        <v>0.006755663733243551</v>
       </c>
     </row>
     <row r="10">
@@ -5003,9 +4999,8 @@
           <t>Std Error (β)</t>
         </is>
       </c>
-      <c r="B10" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!J5:J65,'Monthly Returns'!M5:M65,TRUE,TRUE),2,1)</f>
-        <v/>
+      <c r="B10" s="8" t="n">
+        <v>0.1526967956784597</v>
       </c>
     </row>
     <row r="11">
@@ -5014,9 +5009,8 @@
           <t>t-stat (α)</t>
         </is>
       </c>
-      <c r="B11" s="8">
-        <f>B6/B9</f>
-        <v/>
+      <c r="B11" s="8" t="n">
+        <v>0.5985385833609286</v>
       </c>
     </row>
     <row r="12">
@@ -5025,9 +5019,8 @@
           <t>t-stat (β)</t>
         </is>
       </c>
-      <c r="B12" s="8">
-        <f>B7/B10</f>
-        <v/>
+      <c r="B12" s="8" t="n">
+        <v>6.991490685378866</v>
       </c>
     </row>
     <row r="13">
@@ -5036,9 +5029,8 @@
           <t>F-statistic</t>
         </is>
       </c>
-      <c r="B13" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!J5:J65,'Monthly Returns'!M5:M65,TRUE,TRUE),4,1)</f>
-        <v/>
+      <c r="B13" s="8" t="n">
+        <v>48.88094200373952</v>
       </c>
     </row>
     <row r="14">
@@ -5047,9 +5039,8 @@
           <t>Observations</t>
         </is>
       </c>
-      <c r="B14" s="8">
-        <f>COUNT('Monthly Returns'!J5:J65)</f>
-        <v/>
+      <c r="B14" s="8" t="n">
+        <v>61</v>
       </c>
     </row>
     <row r="15">
@@ -5058,9 +5049,8 @@
           <t>Std Dev of Residuals</t>
         </is>
       </c>
-      <c r="B15" s="8">
-        <f>STDEV.S('Monthly Returns'!Q5:Q65)</f>
-        <v/>
+      <c r="B15" s="8" t="n">
+        <v>0.05140691471372628</v>
       </c>
     </row>
     <row r="16">
@@ -5069,151 +5059,137 @@
           <t>Appraisal Ratio</t>
         </is>
       </c>
-      <c r="B16" s="8">
-        <f>B6/B15</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17"/>
-    <row r="18"/>
+      <c r="B16" s="8" t="n">
+        <v>0.07865722778882751</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>VFIAX Market Model</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Statistic</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
-        <is>
-          <t>VFIAX Market Model</t>
-        </is>
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>Alpha (α)</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="n">
+        <v>0.0008825471722782096</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Statistic</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Beta (β)</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="n">
+        <v>0.9866246762869674</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>Alpha (α)</t>
-        </is>
-      </c>
-      <c r="B21" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!K5:K65,'Monthly Returns'!M5:M65,TRUE,TRUE),1,2)</f>
-        <v/>
+          <t>R-squared</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="n">
+        <v>0.9813883785637134</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>Beta (β)</t>
-        </is>
-      </c>
-      <c r="B22" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!K5:K65,'Monthly Returns'!M5:M65,TRUE,TRUE),1,1)</f>
-        <v/>
+          <t>Std Error (α)</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="n">
+        <v>0.0007825925655779628</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>R-squared</t>
-        </is>
-      </c>
-      <c r="B23" s="8">
-        <f>RSQ('Monthly Returns'!K5:K65,'Monthly Returns'!M5:M65)</f>
-        <v/>
+          <t>Std Error (β)</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="n">
+        <v>0.01768876927628921</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>Std Error (α)</t>
-        </is>
-      </c>
-      <c r="B24" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!K5:K65,'Monthly Returns'!M5:M65,TRUE,TRUE),2,2)</f>
-        <v/>
+          <t>t-stat (α)</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="n">
+        <v>1.127722407669983</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>Std Error (β)</t>
-        </is>
-      </c>
-      <c r="B25" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!K5:K65,'Monthly Returns'!M5:M65,TRUE,TRUE),2,1)</f>
-        <v/>
+          <t>t-stat (β)</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="n">
+        <v>55.77689780879679</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>t-stat (α)</t>
-        </is>
-      </c>
-      <c r="B26" s="8">
-        <f>B21/B24</f>
-        <v/>
+          <t>F-statistic</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="n">
+        <v>3111.062329172958</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>t-stat (β)</t>
-        </is>
-      </c>
-      <c r="B27" s="8">
-        <f>B22/B25</f>
-        <v/>
+          <t>Observations</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="n">
+        <v>61</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>F-statistic</t>
-        </is>
-      </c>
-      <c r="B28" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!K5:K65,'Monthly Returns'!M5:M65,TRUE,TRUE),4,1)</f>
-        <v/>
+          <t>Std Dev of Residuals</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="n">
+        <v>0.00595510239449809</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>Observations</t>
-        </is>
-      </c>
-      <c r="B29" s="8">
-        <f>COUNT('Monthly Returns'!K5:K65)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="7" t="inlineStr">
-        <is>
-          <t>Std Dev of Residuals</t>
-        </is>
-      </c>
-      <c r="B30" s="8">
-        <f>STDEV.S('Monthly Returns'!R5:R65)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="7" t="inlineStr">
-        <is>
           <t>Appraisal Ratio</t>
         </is>
       </c>
-      <c r="B31" s="8">
-        <f>B21/B30</f>
-        <v/>
+      <c r="B29" s="8" t="n">
+        <v>0.1482001674889073</v>
       </c>
     </row>
   </sheetData>
@@ -5281,9 +5257,8 @@
           <t>Alpha (α)</t>
         </is>
       </c>
-      <c r="B6" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!J5:J65,'Monthly Returns'!M5:P65,TRUE,TRUE),1,5)</f>
-        <v/>
+      <c r="B6" s="8" t="n">
+        <v>0.007200433600387687</v>
       </c>
     </row>
     <row r="7">
@@ -5292,9 +5267,8 @@
           <t>β (Mkt-RF)</t>
         </is>
       </c>
-      <c r="B7" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!J5:J65,'Monthly Returns'!M5:P65,TRUE,TRUE),1,4)</f>
-        <v/>
+      <c r="B7" s="8" t="n">
+        <v>0.9485467913274813</v>
       </c>
     </row>
     <row r="8">
@@ -5303,9 +5277,8 @@
           <t>β (SMB)</t>
         </is>
       </c>
-      <c r="B8" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!J5:J65,'Monthly Returns'!M5:P65,TRUE,TRUE),1,3)</f>
-        <v/>
+      <c r="B8" s="8" t="n">
+        <v>-0.176697944717773</v>
       </c>
     </row>
     <row r="9">
@@ -5314,9 +5287,8 @@
           <t>β (HML)</t>
         </is>
       </c>
-      <c r="B9" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!J5:J65,'Monthly Returns'!M5:P65,TRUE,TRUE),1,2)</f>
-        <v/>
+      <c r="B9" s="8" t="n">
+        <v>-0.3405862633375593</v>
       </c>
     </row>
     <row r="10">
@@ -5325,9 +5297,8 @@
           <t>β (Mom)</t>
         </is>
       </c>
-      <c r="B10" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!J5:J65,'Monthly Returns'!M5:P65,TRUE,TRUE),1,1)</f>
-        <v/>
+      <c r="B10" s="8" t="n">
+        <v>-0.4550173476832127</v>
       </c>
     </row>
     <row r="11">
@@ -5336,9 +5307,8 @@
           <t>R-squared</t>
         </is>
       </c>
-      <c r="B11" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!J5:J65,'Monthly Returns'!M5:P65,TRUE,TRUE),3,1)</f>
-        <v/>
+      <c r="B11" s="8" t="n">
+        <v>0.531859040219093</v>
       </c>
     </row>
     <row r="12">
@@ -5347,9 +5317,8 @@
           <t>SE (α)</t>
         </is>
       </c>
-      <c r="B12" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!J5:J65,'Monthly Returns'!M5:P65,TRUE,TRUE),2,5)</f>
-        <v/>
+      <c r="B12" s="8" t="n">
+        <v>0.006759767528709857</v>
       </c>
     </row>
     <row r="13">
@@ -5358,9 +5327,8 @@
           <t>SE (Mkt-RF)</t>
         </is>
       </c>
-      <c r="B13" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!J5:J65,'Monthly Returns'!M5:P65,TRUE,TRUE),2,4)</f>
-        <v/>
+      <c r="B13" s="8" t="n">
+        <v>0.1556779412971221</v>
       </c>
     </row>
     <row r="14">
@@ -5369,9 +5337,8 @@
           <t>SE (SMB)</t>
         </is>
       </c>
-      <c r="B14" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!J5:J65,'Monthly Returns'!M5:P65,TRUE,TRUE),2,3)</f>
-        <v/>
+      <c r="B14" s="8" t="n">
+        <v>0.2491337058813601</v>
       </c>
     </row>
     <row r="15">
@@ -5380,9 +5347,8 @@
           <t>SE (HML)</t>
         </is>
       </c>
-      <c r="B15" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!J5:J65,'Monthly Returns'!M5:P65,TRUE,TRUE),2,2)</f>
-        <v/>
+      <c r="B15" s="8" t="n">
+        <v>0.157066687710358</v>
       </c>
     </row>
     <row r="16">
@@ -5391,9 +5357,8 @@
           <t>SE (Mom)</t>
         </is>
       </c>
-      <c r="B16" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!J5:J65,'Monthly Returns'!M5:P65,TRUE,TRUE),2,1)</f>
-        <v/>
+      <c r="B16" s="8" t="n">
+        <v>0.1925713904124145</v>
       </c>
     </row>
     <row r="17">
@@ -5402,9 +5367,8 @@
           <t>t-stat (α)</t>
         </is>
       </c>
-      <c r="B17" s="8">
-        <f>B6/B12</f>
-        <v/>
+      <c r="B17" s="8" t="n">
+        <v>1.065189530528417</v>
       </c>
     </row>
     <row r="18">
@@ -5413,9 +5377,8 @@
           <t>t-stat (Mkt-RF)</t>
         </is>
       </c>
-      <c r="B18" s="8">
-        <f>B7/B13</f>
-        <v/>
+      <c r="B18" s="8" t="n">
+        <v>6.093007033778241</v>
       </c>
     </row>
     <row r="19">
@@ -5424,9 +5387,8 @@
           <t>t-stat (SMB)</t>
         </is>
       </c>
-      <c r="B19" s="8">
-        <f>B8/B14</f>
-        <v/>
+      <c r="B19" s="8" t="n">
+        <v>-0.7092494533915789</v>
       </c>
     </row>
     <row r="20">
@@ -5435,9 +5397,8 @@
           <t>t-stat (HML)</t>
         </is>
       </c>
-      <c r="B20" s="8">
-        <f>B9/B15</f>
-        <v/>
+      <c r="B20" s="8" t="n">
+        <v>-2.16841819422349</v>
       </c>
     </row>
     <row r="21">
@@ -5446,9 +5407,8 @@
           <t>t-stat (Mom)</t>
         </is>
       </c>
-      <c r="B21" s="8">
-        <f>B10/B16</f>
-        <v/>
+      <c r="B21" s="8" t="n">
+        <v>-2.362850196536148</v>
       </c>
     </row>
     <row r="22">
@@ -5457,9 +5417,8 @@
           <t>F-statistic</t>
         </is>
       </c>
-      <c r="B22" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!J5:J65,'Monthly Returns'!M5:P65,TRUE,TRUE),4,1)</f>
-        <v/>
+      <c r="B22" s="8" t="n">
+        <v>15.905522487398</v>
       </c>
     </row>
     <row r="23">
@@ -5468,9 +5427,8 @@
           <t>Observations</t>
         </is>
       </c>
-      <c r="B23" s="8">
-        <f>COUNT('Monthly Returns'!J5:J65)</f>
-        <v/>
+      <c r="B23" s="8" t="n">
+        <v>61</v>
       </c>
     </row>
     <row r="24"/>
@@ -5500,9 +5458,8 @@
           <t>Alpha (α)</t>
         </is>
       </c>
-      <c r="B28" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!K5:K65,'Monthly Returns'!M5:P65,TRUE,TRUE),1,5)</f>
-        <v/>
+      <c r="B28" s="8" t="n">
+        <v>-0.0003422582669747701</v>
       </c>
     </row>
     <row r="29">
@@ -5511,9 +5468,8 @@
           <t>β (Mkt-RF)</t>
         </is>
       </c>
-      <c r="B29" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!K5:K65,'Monthly Returns'!M5:P65,TRUE,TRUE),1,4)</f>
-        <v/>
+      <c r="B29" s="8" t="n">
+        <v>1.013348486445862</v>
       </c>
     </row>
     <row r="30">
@@ -5522,9 +5478,8 @@
           <t>β (SMB)</t>
         </is>
       </c>
-      <c r="B30" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!K5:K65,'Monthly Returns'!M5:P65,TRUE,TRUE),1,3)</f>
-        <v/>
+      <c r="B30" s="8" t="n">
+        <v>-0.1501017016351763</v>
       </c>
     </row>
     <row r="31">
@@ -5533,9 +5488,8 @@
           <t>β (HML)</t>
         </is>
       </c>
-      <c r="B31" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!K5:K65,'Monthly Returns'!M5:P65,TRUE,TRUE),1,2)</f>
-        <v/>
+      <c r="B31" s="8" t="n">
+        <v>0.03000246040021676</v>
       </c>
     </row>
     <row r="32">
@@ -5544,9 +5498,8 @@
           <t>β (Mom)</t>
         </is>
       </c>
-      <c r="B32" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!K5:K65,'Monthly Returns'!M5:P65,TRUE,TRUE),1,1)</f>
-        <v/>
+      <c r="B32" s="8" t="n">
+        <v>-0.01507942658916988</v>
       </c>
     </row>
     <row r="33">
@@ -5555,9 +5508,8 @@
           <t>R-squared</t>
         </is>
       </c>
-      <c r="B33" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!K5:K65,'Monthly Returns'!M5:P65,TRUE,TRUE),3,1)</f>
-        <v/>
+      <c r="B33" s="8" t="n">
+        <v>0.9899690663830603</v>
       </c>
     </row>
     <row r="34">
@@ -5566,9 +5518,8 @@
           <t>SE (α)</t>
         </is>
       </c>
-      <c r="B34" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!K5:K65,'Monthly Returns'!M5:P65,TRUE,TRUE),2,5)</f>
-        <v/>
+      <c r="B34" s="8" t="n">
+        <v>0.0006213600792786562</v>
       </c>
     </row>
     <row r="35">
@@ -5577,9 +5528,8 @@
           <t>SE (Mkt-RF)</t>
         </is>
       </c>
-      <c r="B35" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!K5:K65,'Monthly Returns'!M5:P65,TRUE,TRUE),2,4)</f>
-        <v/>
+      <c r="B35" s="8" t="n">
+        <v>0.01430996813654917</v>
       </c>
     </row>
     <row r="36">
@@ -5588,9 +5538,8 @@
           <t>SE (SMB)</t>
         </is>
       </c>
-      <c r="B36" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!K5:K65,'Monthly Returns'!M5:P65,TRUE,TRUE),2,3)</f>
-        <v/>
+      <c r="B36" s="8" t="n">
+        <v>0.0229004530969384</v>
       </c>
     </row>
     <row r="37">
@@ -5599,9 +5548,8 @@
           <t>SE (HML)</t>
         </is>
       </c>
-      <c r="B37" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!K5:K65,'Monthly Returns'!M5:P65,TRUE,TRUE),2,2)</f>
-        <v/>
+      <c r="B37" s="8" t="n">
+        <v>0.01443762216869765</v>
       </c>
     </row>
     <row r="38">
@@ -5610,9 +5558,8 @@
           <t>SE (Mom)</t>
         </is>
       </c>
-      <c r="B38" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!K5:K65,'Monthly Returns'!M5:P65,TRUE,TRUE),2,1)</f>
-        <v/>
+      <c r="B38" s="8" t="n">
+        <v>0.01770122624857426</v>
       </c>
     </row>
     <row r="39">
@@ -5621,9 +5568,8 @@
           <t>t-stat (α)</t>
         </is>
       </c>
-      <c r="B39" s="8">
-        <f>B28/B34</f>
-        <v/>
+      <c r="B39" s="8" t="n">
+        <v>-0.5508211396073296</v>
       </c>
     </row>
     <row r="40">
@@ -5632,9 +5578,8 @@
           <t>t-stat (Mkt-RF)</t>
         </is>
       </c>
-      <c r="B40" s="8">
-        <f>B29/B35</f>
-        <v/>
+      <c r="B40" s="8" t="n">
+        <v>70.81416791262187</v>
       </c>
     </row>
     <row r="41">
@@ -5643,9 +5588,8 @@
           <t>t-stat (SMB)</t>
         </is>
       </c>
-      <c r="B41" s="8">
-        <f>B30/B36</f>
-        <v/>
+      <c r="B41" s="8" t="n">
+        <v>-6.55452977282985</v>
       </c>
     </row>
     <row r="42">
@@ -5654,9 +5598,8 @@
           <t>t-stat (HML)</t>
         </is>
       </c>
-      <c r="B42" s="8">
-        <f>B31/B37</f>
-        <v/>
+      <c r="B42" s="8" t="n">
+        <v>2.078074910788661</v>
       </c>
     </row>
     <row r="43">
@@ -5665,9 +5608,8 @@
           <t>t-stat (Mom)</t>
         </is>
       </c>
-      <c r="B43" s="8">
-        <f>B32/B38</f>
-        <v/>
+      <c r="B43" s="8" t="n">
+        <v>-0.8518859867340798</v>
       </c>
     </row>
     <row r="44">
@@ -5676,9 +5618,8 @@
           <t>F-statistic</t>
         </is>
       </c>
-      <c r="B44" s="8">
-        <f>INDEX(LINEST('Monthly Returns'!K5:K65,'Monthly Returns'!M5:P65,TRUE,TRUE),4,1)</f>
-        <v/>
+      <c r="B44" s="8" t="n">
+        <v>1381.682648757396</v>
       </c>
     </row>
     <row r="45">
@@ -5687,9 +5628,8 @@
           <t>Observations</t>
         </is>
       </c>
-      <c r="B45" s="8">
-        <f>COUNT('Monthly Returns'!K5:K65)</f>
-        <v/>
+      <c r="B45" s="8" t="n">
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Final corrections to Excel and Word files
Excel:
- Observations now displays as integer (not 61.0000)
- Alpha/Beta/SE use 6 decimal places for precision
- t-stats/R²/Appraisal use 4 decimal places, F-stat uses 2

Word:
- Fixed VFIAX β(SMB) = -0.1501 (t=-6.55): highly significant at 1%,
  correctly explained as large-cap structural tilt, NOT 'close to zero'
- Fixed VFIAX β(HML) = 0.0300 (t=2.08): significant at 5%, updated text
- Fixed b.2) appraisal ratio: added breakdown table showing alpha and
  residual std dev, corrected explanation of why VFIAX ratio is higher
- Fixed 1.d closing paragraph with actual R² improvement numbers

https://claude.ai/code/session_01UFgKuhfYfoTRdFuN7kHBHu
</commit_message>
<xml_diff>
--- a/Finance_Homework.xlsx
+++ b/Finance_Homework.xlsx
@@ -19,11 +19,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="MMM YYYY"/>
     <numFmt numFmtId="166" formatCode="0.0000%"/>
     <numFmt numFmtId="167" formatCode="0.0000"/>
+    <numFmt numFmtId="168" formatCode="0.000000"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -87,7 +88,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -102,6 +103,8 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -4959,7 +4962,7 @@
           <t>Alpha (α)</t>
         </is>
       </c>
-      <c r="B6" s="8" t="n">
+      <c r="B6" s="12" t="n">
         <v>0.004043525400558397</v>
       </c>
     </row>
@@ -4969,7 +4972,7 @@
           <t>Beta (β)</t>
         </is>
       </c>
-      <c r="B7" s="8" t="n">
+      <c r="B7" s="12" t="n">
         <v>1.067578224673151</v>
       </c>
     </row>
@@ -4989,7 +4992,7 @@
           <t>Std Error (α)</t>
         </is>
       </c>
-      <c r="B9" s="8" t="n">
+      <c r="B9" s="12" t="n">
         <v>0.006755663733243551</v>
       </c>
     </row>
@@ -4999,7 +5002,7 @@
           <t>Std Error (β)</t>
         </is>
       </c>
-      <c r="B10" s="8" t="n">
+      <c r="B10" s="12" t="n">
         <v>0.1526967956784597</v>
       </c>
     </row>
@@ -5029,7 +5032,7 @@
           <t>F-statistic</t>
         </is>
       </c>
-      <c r="B13" s="8" t="n">
+      <c r="B13" s="13" t="n">
         <v>48.88094200373952</v>
       </c>
     </row>
@@ -5039,7 +5042,7 @@
           <t>Observations</t>
         </is>
       </c>
-      <c r="B14" s="8" t="n">
+      <c r="B14" s="9" t="n">
         <v>61</v>
       </c>
     </row>
@@ -5049,7 +5052,7 @@
           <t>Std Dev of Residuals</t>
         </is>
       </c>
-      <c r="B15" s="8" t="n">
+      <c r="B15" s="12" t="n">
         <v>0.05140691471372628</v>
       </c>
     </row>
@@ -5088,7 +5091,7 @@
           <t>Alpha (α)</t>
         </is>
       </c>
-      <c r="B19" s="8" t="n">
+      <c r="B19" s="12" t="n">
         <v>0.0008825471722782096</v>
       </c>
     </row>
@@ -5098,7 +5101,7 @@
           <t>Beta (β)</t>
         </is>
       </c>
-      <c r="B20" s="8" t="n">
+      <c r="B20" s="12" t="n">
         <v>0.9866246762869674</v>
       </c>
     </row>
@@ -5118,7 +5121,7 @@
           <t>Std Error (α)</t>
         </is>
       </c>
-      <c r="B22" s="8" t="n">
+      <c r="B22" s="12" t="n">
         <v>0.0007825925655779628</v>
       </c>
     </row>
@@ -5128,7 +5131,7 @@
           <t>Std Error (β)</t>
         </is>
       </c>
-      <c r="B23" s="8" t="n">
+      <c r="B23" s="12" t="n">
         <v>0.01768876927628921</v>
       </c>
     </row>
@@ -5158,7 +5161,7 @@
           <t>F-statistic</t>
         </is>
       </c>
-      <c r="B26" s="8" t="n">
+      <c r="B26" s="13" t="n">
         <v>3111.062329172958</v>
       </c>
     </row>
@@ -5168,7 +5171,7 @@
           <t>Observations</t>
         </is>
       </c>
-      <c r="B27" s="8" t="n">
+      <c r="B27" s="9" t="n">
         <v>61</v>
       </c>
     </row>
@@ -5178,7 +5181,7 @@
           <t>Std Dev of Residuals</t>
         </is>
       </c>
-      <c r="B28" s="8" t="n">
+      <c r="B28" s="12" t="n">
         <v>0.00595510239449809</v>
       </c>
     </row>
@@ -5257,7 +5260,7 @@
           <t>Alpha (α)</t>
         </is>
       </c>
-      <c r="B6" s="8" t="n">
+      <c r="B6" s="12" t="n">
         <v>0.007200433600387687</v>
       </c>
     </row>
@@ -5267,7 +5270,7 @@
           <t>β (Mkt-RF)</t>
         </is>
       </c>
-      <c r="B7" s="8" t="n">
+      <c r="B7" s="12" t="n">
         <v>0.9485467913274813</v>
       </c>
     </row>
@@ -5277,7 +5280,7 @@
           <t>β (SMB)</t>
         </is>
       </c>
-      <c r="B8" s="8" t="n">
+      <c r="B8" s="12" t="n">
         <v>-0.176697944717773</v>
       </c>
     </row>
@@ -5287,7 +5290,7 @@
           <t>β (HML)</t>
         </is>
       </c>
-      <c r="B9" s="8" t="n">
+      <c r="B9" s="12" t="n">
         <v>-0.3405862633375593</v>
       </c>
     </row>
@@ -5297,7 +5300,7 @@
           <t>β (Mom)</t>
         </is>
       </c>
-      <c r="B10" s="8" t="n">
+      <c r="B10" s="12" t="n">
         <v>-0.4550173476832127</v>
       </c>
     </row>
@@ -5317,7 +5320,7 @@
           <t>SE (α)</t>
         </is>
       </c>
-      <c r="B12" s="8" t="n">
+      <c r="B12" s="12" t="n">
         <v>0.006759767528709857</v>
       </c>
     </row>
@@ -5327,7 +5330,7 @@
           <t>SE (Mkt-RF)</t>
         </is>
       </c>
-      <c r="B13" s="8" t="n">
+      <c r="B13" s="12" t="n">
         <v>0.1556779412971221</v>
       </c>
     </row>
@@ -5337,7 +5340,7 @@
           <t>SE (SMB)</t>
         </is>
       </c>
-      <c r="B14" s="8" t="n">
+      <c r="B14" s="12" t="n">
         <v>0.2491337058813601</v>
       </c>
     </row>
@@ -5347,7 +5350,7 @@
           <t>SE (HML)</t>
         </is>
       </c>
-      <c r="B15" s="8" t="n">
+      <c r="B15" s="12" t="n">
         <v>0.157066687710358</v>
       </c>
     </row>
@@ -5357,7 +5360,7 @@
           <t>SE (Mom)</t>
         </is>
       </c>
-      <c r="B16" s="8" t="n">
+      <c r="B16" s="12" t="n">
         <v>0.1925713904124145</v>
       </c>
     </row>
@@ -5417,7 +5420,7 @@
           <t>F-statistic</t>
         </is>
       </c>
-      <c r="B22" s="8" t="n">
+      <c r="B22" s="13" t="n">
         <v>15.905522487398</v>
       </c>
     </row>
@@ -5427,7 +5430,7 @@
           <t>Observations</t>
         </is>
       </c>
-      <c r="B23" s="8" t="n">
+      <c r="B23" s="9" t="n">
         <v>61</v>
       </c>
     </row>
@@ -5458,7 +5461,7 @@
           <t>Alpha (α)</t>
         </is>
       </c>
-      <c r="B28" s="8" t="n">
+      <c r="B28" s="12" t="n">
         <v>-0.0003422582669747701</v>
       </c>
     </row>
@@ -5468,7 +5471,7 @@
           <t>β (Mkt-RF)</t>
         </is>
       </c>
-      <c r="B29" s="8" t="n">
+      <c r="B29" s="12" t="n">
         <v>1.013348486445862</v>
       </c>
     </row>
@@ -5478,7 +5481,7 @@
           <t>β (SMB)</t>
         </is>
       </c>
-      <c r="B30" s="8" t="n">
+      <c r="B30" s="12" t="n">
         <v>-0.1501017016351763</v>
       </c>
     </row>
@@ -5488,7 +5491,7 @@
           <t>β (HML)</t>
         </is>
       </c>
-      <c r="B31" s="8" t="n">
+      <c r="B31" s="12" t="n">
         <v>0.03000246040021676</v>
       </c>
     </row>
@@ -5498,7 +5501,7 @@
           <t>β (Mom)</t>
         </is>
       </c>
-      <c r="B32" s="8" t="n">
+      <c r="B32" s="12" t="n">
         <v>-0.01507942658916988</v>
       </c>
     </row>
@@ -5518,7 +5521,7 @@
           <t>SE (α)</t>
         </is>
       </c>
-      <c r="B34" s="8" t="n">
+      <c r="B34" s="12" t="n">
         <v>0.0006213600792786562</v>
       </c>
     </row>
@@ -5528,7 +5531,7 @@
           <t>SE (Mkt-RF)</t>
         </is>
       </c>
-      <c r="B35" s="8" t="n">
+      <c r="B35" s="12" t="n">
         <v>0.01430996813654917</v>
       </c>
     </row>
@@ -5538,7 +5541,7 @@
           <t>SE (SMB)</t>
         </is>
       </c>
-      <c r="B36" s="8" t="n">
+      <c r="B36" s="12" t="n">
         <v>0.0229004530969384</v>
       </c>
     </row>
@@ -5548,7 +5551,7 @@
           <t>SE (HML)</t>
         </is>
       </c>
-      <c r="B37" s="8" t="n">
+      <c r="B37" s="12" t="n">
         <v>0.01443762216869765</v>
       </c>
     </row>
@@ -5558,7 +5561,7 @@
           <t>SE (Mom)</t>
         </is>
       </c>
-      <c r="B38" s="8" t="n">
+      <c r="B38" s="12" t="n">
         <v>0.01770122624857426</v>
       </c>
     </row>
@@ -5618,7 +5621,7 @@
           <t>F-statistic</t>
         </is>
       </c>
-      <c r="B44" s="8" t="n">
+      <c r="B44" s="13" t="n">
         <v>1381.682648757396</v>
       </c>
     </row>
@@ -5628,7 +5631,7 @@
           <t>Observations</t>
         </is>
       </c>
-      <c r="B45" s="8" t="n">
+      <c r="B45" s="9" t="n">
         <v>61</v>
       </c>
     </row>

</xml_diff>